<commit_message>
Store TOEFL minimums on both the 0-120 and the 2026 1-6 band scale
The TOEFL iBT moved to a 1-6 band scale on 21 January 2026, with 0-120
reported alongside only during a two-year transition, so universities now
publish minimums on either scale. course.toefl_2026 (DECIMAL(2,1), 1-6)
sits beside the existing toefl (0-120), via migration 20261006140000.

- Program form: "TOEFL iBT 2026 (1-6)" field; validated 1-6 in 0.5 steps.
- Bulk import: toefl_2026 column, same validation (a 0-120 score there is
  a row error, which catches a column mix-up).
- Uni Assist: new "TOEFL iBT 2026 (1-6)" test option, compared against
  toefl_2026; the 0-120 option keeps using toefl. A program that states only
  the other scale counts as stating no requirement, as with any test.
- Template and the TCD worked example carry both columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/University_Course_Import_Template.xlsx
+++ b/docs/University_Course_Import_Template.xlsx
@@ -493,7 +493,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AD2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -506,24 +506,25 @@
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
     <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
     <col min="13" max="13" width="10.83203125" customWidth="1"/>
     <col min="14" max="14" width="10.83203125" customWidth="1"/>
     <col min="15" max="15" width="10.83203125" customWidth="1"/>
     <col min="16" max="16" width="10.83203125" customWidth="1"/>
-    <col min="17" max="17" width="22.83203125" customWidth="1"/>
-    <col min="18" max="18" width="10.83203125" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" customWidth="1"/>
-    <col min="20" max="20" width="13.83203125" customWidth="1"/>
-    <col min="21" max="21" width="19.83203125" customWidth="1"/>
-    <col min="22" max="22" width="20.83203125" customWidth="1"/>
-    <col min="23" max="23" width="10.83203125" customWidth="1"/>
-    <col min="24" max="24" width="21.83203125" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
-    <col min="26" max="26" width="20.83203125" customWidth="1"/>
-    <col min="27" max="27" width="24.83203125" customWidth="1"/>
-    <col min="28" max="28" width="30.83203125" customWidth="1"/>
-    <col min="29" max="29" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="10.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="13.83203125" customWidth="1"/>
+    <col min="22" max="22" width="19.83203125" customWidth="1"/>
+    <col min="23" max="23" width="20.83203125" customWidth="1"/>
+    <col min="24" max="24" width="10.83203125" customWidth="1"/>
+    <col min="25" max="25" width="21.83203125" customWidth="1"/>
+    <col min="26" max="26" width="17.83203125" customWidth="1"/>
+    <col min="27" max="27" width="20.83203125" customWidth="1"/>
+    <col min="28" max="28" width="24.83203125" customWidth="1"/>
+    <col min="29" max="29" width="30.83203125" customWidth="1"/>
+    <col min="30" max="30" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,57 +562,60 @@
         <v>toefl</v>
       </c>
       <c r="L1" t="str">
+        <v>toefl_2026</v>
+      </c>
+      <c r="M1" t="str">
         <v>ielts</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>det</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>pte</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>gre</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>gmat</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>application_deadline</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>is_stem</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>intake_month</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>intake_year</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>is_coop_available</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>has_app_fee_waiver</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>app_fee</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>has_tuition_deposit</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>has_scholarship</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>scholarship_amount</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>min_entry_requirements</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>min_entry_requirements_scale</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>has_faster_tat</v>
       </c>
     </row>
@@ -646,74 +650,77 @@
       <c r="J2" t="str">
         <v>Yes</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
+      <c r="K2">
+        <v>90</v>
       </c>
       <c r="L2">
+        <v>4.5</v>
+      </c>
+      <c r="M2">
         <v>6.5</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>120</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>69</v>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
       <c r="P2" t="str">
         <v/>
       </c>
       <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v>2027-06-30</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v>No</v>
       </c>
-      <c r="S2" t="str">
+      <c r="T2" t="str">
         <v>Sep</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>2027</v>
-      </c>
-      <c r="U2" t="str">
-        <v>No</v>
       </c>
       <c r="V2" t="str">
         <v>No</v>
       </c>
-      <c r="W2">
+      <c r="W2" t="str">
+        <v>No</v>
+      </c>
+      <c r="X2">
         <v>55</v>
-      </c>
-      <c r="X2" t="str">
-        <v>Yes</v>
       </c>
       <c r="Y2" t="str">
         <v>Yes</v>
       </c>
-      <c r="Z2">
+      <c r="Z2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA2">
         <v>2000</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AB2" t="str">
         <v>An upper second-class (2.1) Honours degree or higher in Computing or a related discipline, plus proven programming competence.</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AC2" t="str">
         <v>UK honours</v>
       </c>
-      <c r="AC2" t="str">
+      <c r="AD2" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -945,26 +952,37 @@
         <v>toefl</v>
       </c>
       <c r="B21" t="str">
-        <v>Number</v>
+        <v>Number, 0-120</v>
       </c>
       <c r="C21" t="str">
-        <v>TOEFL iBT minimum on the 0-120 scale (see the guide on the 2026 1-6 band scale).</v>
+        <v>TOEFL iBT minimum on the 0-120 scale (the test before January 2026, and the comparable score reported during the transition).</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>toefl_2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>1 to 6, in steps of 0.5</v>
+      </c>
+      <c r="C22" t="str">
+        <v>TOEFL iBT minimum on the 2026 band scale. Fill both when the university states both; ETS equivalents: 4 = 80, 4.5 = 90, 5 = 100.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>min_entry_requirements_scale</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B23" t="str">
         <v>Max 20 characters</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C23" t="str">
         <v>The scale for the value above, e.g. UK honours, 4.0 GPA, %</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>